<commit_message>
minor change to v18 long
</commit_message>
<xml_diff>
--- a/www/data-entry-template/GLATAR_data_entry_template_v18_long.xlsx
+++ b/www/data-entry-template/GLATAR_data_entry_template_v18_long.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benhlina/Library/CloudStorage/Dropbox/GitHub/GLATAR-App/www/data-entry-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E7419FD-2AC0-3E4B-B4EA-EF049FF0EF06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A4463F4-9383-E848-B007-BB06C04B1C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19000" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19000" activeTab="3" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
   </bookViews>
   <sheets>
     <sheet name="data_dictionary" sheetId="1" r:id="rId1"/>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="292">
   <si>
     <t>Field Name</t>
   </si>
@@ -1168,16 +1168,7 @@
     <t>thiamine_type</t>
   </si>
   <si>
-    <t>thiamine_nmol_g_sd</t>
-  </si>
-  <si>
     <t>thiaminase_activity</t>
-  </si>
-  <si>
-    <t>thiaminase_activity_sd</t>
-  </si>
-  <si>
-    <t>Standard deviation of Thiamine measurment if reported as mean</t>
   </si>
   <si>
     <t>Vitamer type (e.g., Th (free thiamine), TMP (thiamine monophosphate), TPP (thiamine pyrophosphate), and TTh (total thiamine))</t>
@@ -1192,13 +1183,7 @@
     <t>as in: 0.6; format: numeric</t>
   </si>
   <si>
-    <t>as in: 0.02; fromat: numeric</t>
-  </si>
-  <si>
     <t xml:space="preserve">Thiaminase activity measured in unit xxx </t>
-  </si>
-  <si>
-    <t>Standard deviation of Thiaminase activity if reported as mean</t>
   </si>
   <si>
     <t>as in: Alanine; format: character</t>
@@ -1214,9 +1199,6 @@
   </si>
   <si>
     <t>as in: 2.4 ‰; format: numeric</t>
-  </si>
-  <si>
-    <t>as in: 0.12; format: numeric</t>
   </si>
   <si>
     <t>data_type</t>
@@ -1923,7 +1905,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCDB0B4B-8041-E244-B061-95D35DE0CD3B}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D92"/>
+  <dimension ref="A1:D90"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" style="1" customWidth="1"/>
@@ -2472,13 +2454,13 @@
         <v>137</v>
       </c>
       <c r="B41" s="30" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="C41" s="30" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="D41" s="33" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
@@ -2486,7 +2468,7 @@
         <v>137</v>
       </c>
       <c r="B42" s="30" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="C42" s="30" t="s">
         <v>72</v>
@@ -3021,7 +3003,7 @@
         <v>245</v>
       </c>
       <c r="C80" s="30" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="D80" s="33" t="s">
         <v>246</v>
@@ -3049,7 +3031,7 @@
         <v>249</v>
       </c>
       <c r="C82" s="30" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="D82" s="33" t="s">
         <v>250</v>
@@ -3063,66 +3045,66 @@
         <v>251</v>
       </c>
       <c r="C83" s="30" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="D83" s="30" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="84" spans="1:4" ht="28" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:4" ht="42" x14ac:dyDescent="0.2">
       <c r="A84" s="30" t="s">
         <v>266</v>
       </c>
       <c r="B84" s="40" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C84" s="30" t="s">
-        <v>293</v>
+        <v>280</v>
       </c>
       <c r="D84" s="33" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85" s="30" t="s">
         <v>266</v>
       </c>
       <c r="B85" s="40" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C85" s="30" t="s">
-        <v>283</v>
-      </c>
-      <c r="D85" s="33" t="s">
         <v>281</v>
+      </c>
+      <c r="D85" s="30" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" s="30" t="s">
-        <v>266</v>
-      </c>
-      <c r="B86" s="40" t="s">
-        <v>278</v>
+        <v>264</v>
+      </c>
+      <c r="B86" s="30" t="s">
+        <v>253</v>
       </c>
       <c r="C86" s="30" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D86" s="30" t="s">
-        <v>286</v>
+        <v>254</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A87" s="30" t="s">
-        <v>266</v>
-      </c>
-      <c r="B87" s="40" t="s">
-        <v>279</v>
+        <v>264</v>
+      </c>
+      <c r="B87" s="30" t="s">
+        <v>255</v>
       </c>
       <c r="C87" s="30" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D87" s="30" t="s">
-        <v>287</v>
+        <v>256</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
@@ -3130,13 +3112,13 @@
         <v>264</v>
       </c>
       <c r="B88" s="30" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
       <c r="C88" s="30" t="s">
-        <v>290</v>
+        <v>257</v>
       </c>
       <c r="D88" s="30" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
@@ -3144,13 +3126,13 @@
         <v>264</v>
       </c>
       <c r="B89" s="30" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C89" s="30" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="D89" s="30" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
@@ -3158,40 +3140,12 @@
         <v>264</v>
       </c>
       <c r="B90" s="30" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="C90" s="30" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="D90" s="30" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A91" s="30" t="s">
-        <v>264</v>
-      </c>
-      <c r="B91" s="30" t="s">
-        <v>259</v>
-      </c>
-      <c r="C91" s="30" t="s">
-        <v>291</v>
-      </c>
-      <c r="D91" s="30" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A92" s="30" t="s">
-        <v>264</v>
-      </c>
-      <c r="B92" s="30" t="s">
-        <v>261</v>
-      </c>
-      <c r="C92" s="30" t="s">
-        <v>262</v>
-      </c>
-      <c r="D92" s="30" t="s">
         <v>263</v>
       </c>
     </row>
@@ -44260,7 +44214,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED99CF4A-5D49-794D-A1CB-3B08F37AF445}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:BT14"/>
+  <dimension ref="A1:BR14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.5" customWidth="1"/>
@@ -44301,18 +44255,16 @@
     <col min="60" max="60" width="21.83203125" bestFit="1" customWidth="1"/>
     <col min="61" max="61" width="13.83203125" bestFit="1" customWidth="1"/>
     <col min="62" max="63" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="14.33203125" customWidth="1"/>
-    <col min="66" max="66" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="14.33203125" customWidth="1"/>
+    <col min="65" max="65" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="16.83203125" bestFit="1" customWidth="1"/>
     <col min="69" max="69" width="17.5" bestFit="1" customWidth="1"/>
     <col min="70" max="70" width="16.83203125" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="16.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:72" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:70" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="49" t="s">
         <v>185</v>
       </c>
@@ -44322,7 +44274,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="2" spans="1:72" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A2" s="49" t="s">
         <v>24</v>
       </c>
@@ -44330,7 +44282,7 @@
       <c r="C2" s="50"/>
       <c r="D2" s="6"/>
     </row>
-    <row r="3" spans="1:72" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A3" s="49"/>
       <c r="B3" s="50"/>
       <c r="C3" s="50"/>
@@ -44338,7 +44290,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:72" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>137</v>
       </c>
@@ -44374,17 +44326,15 @@
       </c>
       <c r="BL4" s="38"/>
       <c r="BM4" s="38"/>
-      <c r="BN4" s="38"/>
+      <c r="BN4" s="38" t="s">
+        <v>264</v>
+      </c>
       <c r="BO4" s="38"/>
-      <c r="BP4" s="38" t="s">
-        <v>264</v>
-      </c>
+      <c r="BP4" s="38"/>
       <c r="BQ4" s="38"/>
       <c r="BR4" s="38"/>
-      <c r="BS4" s="38"/>
-      <c r="BT4" s="38"/>
-    </row>
-    <row r="5" spans="1:72" s="4" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:70" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="42" t="s">
         <v>14</v>
       </c>
@@ -44443,10 +44393,10 @@
         <v>197</v>
       </c>
       <c r="T5" s="46" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="U5" s="45" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="V5" s="44" t="s">
         <v>9</v>
@@ -44575,43 +44525,37 @@
         <v>251</v>
       </c>
       <c r="BL5" s="39" t="s">
+        <v>276</v>
+      </c>
+      <c r="BM5" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="BM5" s="39" t="s">
-        <v>276</v>
-      </c>
       <c r="BN5" s="39" t="s">
-        <v>278</v>
+        <v>253</v>
       </c>
       <c r="BO5" s="39" t="s">
-        <v>279</v>
+        <v>255</v>
       </c>
       <c r="BP5" s="39" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
       <c r="BQ5" s="39" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="BR5" s="39" t="s">
-        <v>265</v>
-      </c>
-      <c r="BS5" s="39" t="s">
-        <v>259</v>
-      </c>
-      <c r="BT5" s="39" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="11" spans="1:72" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:70" x14ac:dyDescent="0.2">
       <c r="BK11" s="41"/>
     </row>
-    <row r="12" spans="1:72" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:70" x14ac:dyDescent="0.2">
       <c r="BK12" s="41"/>
     </row>
-    <row r="13" spans="1:72" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:70" x14ac:dyDescent="0.2">
       <c r="BK13" s="41"/>
     </row>
-    <row r="14" spans="1:72" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:70" x14ac:dyDescent="0.2">
       <c r="BK14" s="41"/>
     </row>
   </sheetData>
@@ -44669,7 +44613,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BJ6:BJ9992" xr:uid="{2FF93C04-BFBA-A042-839F-6119E2726FB2}">
       <formula1>"Alanine, Arginine, Aspartic acid, Cysteine, Cystine, Glutamic acid, Glycine, Histidine, Isoleucine, Leucine, Lysine, Methionine, Phenylalanine, Proline, Serine, Threonine, Tyrosine, Valine"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BM6:BM9992" xr:uid="{73E98200-DF79-B04A-8673-08ACB9A22C3B}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL6:BL9992" xr:uid="{73E98200-DF79-B04A-8673-08ACB9A22C3B}">
       <formula1>"Th (free thiamine), TMP (thiamine monophosphate), TPP (thiamine pyrophosphate), TTh (total thiamine)"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V6:V992" xr:uid="{46AB659B-2A50-3441-8038-5315F30CB679}">
@@ -44678,7 +44622,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T6:T10000" xr:uid="{51C4B292-4D0C-024D-B22F-A10ACA6AD19D}">
       <formula1>"Individual, Composite, Mean, SD, Equation"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BQ6:BQ10000" xr:uid="{7BF0785F-9FED-164D-B36A-ADDD49066DAC}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BO6:BO10000" xr:uid="{7BF0785F-9FED-164D-B36A-ADDD49066DAC}">
       <formula1>" total, methyl "</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU6:AU10000" xr:uid="{0C3C69BE-9F3E-1B4B-A562-52BCC53E43F8}">

</xml_diff>